<commit_message>
feat: Update scrape configuration and enhance source handling for improved data extraction
</commit_message>
<xml_diff>
--- a/excel_reports/funding-funnel-report-20260526-092725.xlsx
+++ b/excel_reports/funding-funnel-report-20260526-092725.xlsx
@@ -497,136 +497,140 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="12" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="12" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="13" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="13" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="14" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="14" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="15" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="15" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="15" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="15" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="15" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="15" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="15" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="15" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -952,750 +956,742 @@
   <dimension ref="A1:N24"/>
   <sheetFormatPr defaultColWidth="8.5078125" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="29.49"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="24.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="44.94"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="14.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="15.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="11.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="12.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="14.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42.01"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="27.96"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="21.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="24.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="18.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="44.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="16.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="14.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="15.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="11.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="12.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="14.83"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="70.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
-      <c r="L3" s="3"/>
-      <c r="M3" s="3"/>
-      <c r="N3" s="3"/>
+      <c r="A3" s="4"/>
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3"/>
-      <c r="E4" s="4" t="s">
+      <c r="D4" s="4"/>
+      <c r="E4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
-      <c r="M4" s="4"/>
-      <c r="N4" s="4"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="5"/>
+      <c r="L4" s="5"/>
+      <c r="M4" s="5"/>
+      <c r="N4" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="3"/>
-      <c r="E5" s="8" t="s">
+      <c r="D5" s="4"/>
+      <c r="E5" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="8"/>
-      <c r="G5" s="8"/>
-      <c r="H5" s="8"/>
-      <c r="I5" s="8"/>
-      <c r="J5" s="8"/>
-      <c r="K5" s="8"/>
-      <c r="L5" s="8"/>
-      <c r="M5" s="8"/>
-      <c r="N5" s="8"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
+      <c r="N5" s="9"/>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="10" t="n">
+      <c r="B6" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="3"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="8"/>
-      <c r="K6" s="8"/>
-      <c r="L6" s="8"/>
-      <c r="M6" s="8"/>
-      <c r="N6" s="8"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="9"/>
+      <c r="L6" s="9"/>
+      <c r="M6" s="9"/>
+      <c r="N6" s="9"/>
     </row>
     <row r="7" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="13" t="n">
+      <c r="B7" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="3"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="8"/>
-      <c r="L7" s="8"/>
-      <c r="M7" s="8"/>
-      <c r="N7" s="8"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="9"/>
+      <c r="M7" s="9"/>
+      <c r="N7" s="9"/>
     </row>
     <row r="8" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="14" t="n">
+      <c r="B8" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="3"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
-      <c r="K8" s="8"/>
-      <c r="L8" s="8"/>
-      <c r="M8" s="8"/>
-      <c r="N8" s="8"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
+      <c r="I8" s="9"/>
+      <c r="J8" s="9"/>
+      <c r="K8" s="9"/>
+      <c r="L8" s="9"/>
+      <c r="M8" s="9"/>
+      <c r="N8" s="9"/>
     </row>
     <row r="9" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="16" t="n">
+      <c r="B9" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
-      <c r="M9" s="3"/>
-      <c r="N9" s="3"/>
-    </row>
-    <row r="10" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="17" t="s">
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="4"/>
+      <c r="I9" s="4"/>
+      <c r="J9" s="4"/>
+      <c r="K9" s="4"/>
+      <c r="L9" s="4"/>
+      <c r="M9" s="4"/>
+      <c r="N9" s="4"/>
+    </row>
+    <row r="10" customFormat="false" ht="44.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="18" t="n">
+      <c r="B10" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="3"/>
-      <c r="E10" s="19" t="s">
+      <c r="D10" s="4"/>
+      <c r="E10" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="F10" s="19"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="20" t="s">
+      <c r="F10" s="20"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="I10" s="20"/>
-      <c r="J10" s="20"/>
-      <c r="K10" s="20"/>
-      <c r="L10" s="20"/>
-      <c r="M10" s="20"/>
-      <c r="N10" s="20"/>
+      <c r="I10" s="21"/>
+      <c r="J10" s="21"/>
+      <c r="K10" s="21"/>
+      <c r="L10" s="21"/>
+      <c r="M10" s="21"/>
+      <c r="N10" s="21"/>
     </row>
     <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="s">
+      <c r="A11" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="21" t="n">
+      <c r="B11" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="3"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="20"/>
-      <c r="I11" s="20"/>
-      <c r="J11" s="20"/>
-      <c r="K11" s="20"/>
-      <c r="L11" s="20"/>
-      <c r="M11" s="20"/>
-      <c r="N11" s="20"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="20"/>
+      <c r="F11" s="20"/>
+      <c r="G11" s="4"/>
+      <c r="H11" s="21"/>
+      <c r="I11" s="21"/>
+      <c r="J11" s="21"/>
+      <c r="K11" s="21"/>
+      <c r="L11" s="21"/>
+      <c r="M11" s="21"/>
+      <c r="N11" s="21"/>
     </row>
     <row r="12" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17" t="s">
+      <c r="A12" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="B12" s="22" t="n">
+      <c r="B12" s="23" t="n">
         <v>4580000</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="D12" s="3"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="20"/>
-      <c r="I12" s="20"/>
-      <c r="J12" s="20"/>
-      <c r="K12" s="20"/>
-      <c r="L12" s="20"/>
-      <c r="M12" s="20"/>
-      <c r="N12" s="20"/>
-    </row>
-    <row r="13" customFormat="false" ht="8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="D12" s="4"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="21"/>
+      <c r="I12" s="21"/>
+      <c r="J12" s="21"/>
+      <c r="K12" s="21"/>
+      <c r="L12" s="21"/>
+      <c r="M12" s="21"/>
+      <c r="N12" s="21"/>
+    </row>
+    <row r="13" customFormat="false" ht="46.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="3" t="n">
+      <c r="B13" s="24" t="n">
         <v>458000</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-      <c r="L13" s="3"/>
-      <c r="M13" s="3"/>
-      <c r="N13" s="3"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="4"/>
+      <c r="K13" s="4"/>
+      <c r="L13" s="4"/>
+      <c r="M13" s="4"/>
+      <c r="N13" s="4"/>
     </row>
     <row r="14" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
-      <c r="J14" s="4"/>
-      <c r="K14" s="4"/>
-      <c r="L14" s="4"/>
-      <c r="M14" s="4"/>
-      <c r="N14" s="4"/>
+      <c r="A14" s="5"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+      <c r="I14" s="5"/>
+      <c r="J14" s="5"/>
+      <c r="K14" s="5"/>
+      <c r="L14" s="5"/>
+      <c r="M14" s="5"/>
+      <c r="N14" s="5"/>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="E15" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="F15" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="G15" s="3" t="s">
+      <c r="G15" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="H15" s="23" t="s">
+      <c r="H15" s="25" t="s">
         <v>34</v>
       </c>
-      <c r="I15" s="3" t="s">
+      <c r="I15" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="J15" s="24" t="s">
+      <c r="J15" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="K15" s="25" t="s">
+      <c r="K15" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="L15" s="25" t="s">
+      <c r="L15" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="M15" s="26" t="s">
+      <c r="M15" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="N15" s="25" t="s">
+      <c r="N15" s="24" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="27" t="s">
+      <c r="A16" s="28" t="s">
         <v>40</v>
       </c>
-      <c r="B16" s="28" t="s">
+      <c r="B16" s="29" t="s">
         <v>41</v>
       </c>
-      <c r="C16" s="28" t="s">
+      <c r="C16" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="D16" s="28" t="s">
+      <c r="D16" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="E16" s="28" t="s">
+      <c r="E16" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="F16" s="28" t="s">
+      <c r="F16" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="G16" s="27" t="s">
+      <c r="G16" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="H16" s="29" t="s">
+      <c r="H16" s="30" t="s">
         <v>47</v>
       </c>
-      <c r="I16" s="27" t="s">
+      <c r="I16" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="J16" s="30" t="n">
+      <c r="J16" s="31" t="n">
         <v>250000</v>
       </c>
-      <c r="K16" s="31" t="s">
+      <c r="K16" s="32" t="s">
         <v>49</v>
       </c>
-      <c r="L16" s="32" t="s">
+      <c r="L16" s="33" t="s">
         <v>50</v>
       </c>
-      <c r="M16" s="26" t="s">
+      <c r="M16" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="N16" s="32"/>
+      <c r="N16" s="33"/>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B17" s="28" t="s">
+      <c r="B17" s="29" t="s">
         <v>41</v>
       </c>
-      <c r="C17" s="28" t="s">
+      <c r="C17" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="D17" s="28" t="s">
+      <c r="D17" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="E17" s="28" t="s">
+      <c r="E17" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="F17" s="28" t="s">
+      <c r="F17" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="G17" s="3" t="s">
+      <c r="G17" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="H17" s="23" t="s">
+      <c r="H17" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="I17" s="3" t="s">
+      <c r="I17" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="J17" s="24" t="n">
+      <c r="J17" s="26" t="n">
         <v>50000</v>
       </c>
-      <c r="K17" s="31" t="s">
+      <c r="K17" s="32" t="s">
         <v>49</v>
       </c>
-      <c r="L17" s="25" t="s">
+      <c r="L17" s="24" t="s">
         <v>50</v>
       </c>
-      <c r="M17" s="26" t="s">
+      <c r="M17" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="N17" s="25"/>
+      <c r="N17" s="24"/>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="27" t="s">
+      <c r="A18" s="28" t="s">
         <v>53</v>
       </c>
-      <c r="B18" s="28" t="s">
+      <c r="B18" s="29" t="s">
         <v>41</v>
       </c>
-      <c r="C18" s="28" t="s">
+      <c r="C18" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="D18" s="28" t="s">
+      <c r="D18" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="E18" s="28" t="s">
+      <c r="E18" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="F18" s="28" t="s">
+      <c r="F18" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="G18" s="27" t="s">
+      <c r="G18" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="H18" s="29" t="s">
+      <c r="H18" s="30" t="s">
         <v>54</v>
       </c>
-      <c r="I18" s="27" t="s">
+      <c r="I18" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="J18" s="30" t="n">
+      <c r="J18" s="31" t="n">
         <v>50000</v>
       </c>
-      <c r="K18" s="31" t="s">
+      <c r="K18" s="32" t="s">
         <v>49</v>
       </c>
-      <c r="L18" s="32" t="s">
+      <c r="L18" s="33" t="s">
         <v>50</v>
       </c>
-      <c r="M18" s="26" t="s">
+      <c r="M18" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="N18" s="32"/>
+      <c r="N18" s="33"/>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="28" t="s">
+      <c r="B19" s="29" t="s">
         <v>41</v>
       </c>
-      <c r="C19" s="28" t="s">
+      <c r="C19" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="D19" s="28" t="s">
+      <c r="D19" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="E19" s="28" t="s">
+      <c r="E19" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="F19" s="28" t="s">
+      <c r="F19" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="G19" s="3" t="s">
+      <c r="G19" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="H19" s="23" t="s">
+      <c r="H19" s="25" t="s">
         <v>56</v>
       </c>
-      <c r="I19" s="3" t="s">
+      <c r="I19" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="J19" s="24" t="n">
+      <c r="J19" s="26" t="n">
         <v>100000</v>
       </c>
-      <c r="K19" s="31" t="s">
+      <c r="K19" s="32" t="s">
         <v>49</v>
       </c>
-      <c r="L19" s="25" t="s">
+      <c r="L19" s="24" t="s">
         <v>50</v>
       </c>
-      <c r="M19" s="26" t="s">
+      <c r="M19" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="N19" s="25"/>
+      <c r="N19" s="24"/>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="27" t="s">
+      <c r="A20" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="B20" s="28" t="s">
+      <c r="B20" s="29" t="s">
         <v>41</v>
       </c>
-      <c r="C20" s="28" t="s">
+      <c r="C20" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="D20" s="28" t="s">
+      <c r="D20" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="E20" s="28" t="s">
+      <c r="E20" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="F20" s="28" t="s">
+      <c r="F20" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="G20" s="27" t="s">
+      <c r="G20" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="H20" s="29" t="s">
+      <c r="H20" s="30" t="s">
         <v>58</v>
       </c>
-      <c r="I20" s="27" t="s">
+      <c r="I20" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="J20" s="30" t="n">
+      <c r="J20" s="31" t="n">
         <v>500000</v>
       </c>
-      <c r="K20" s="31" t="s">
+      <c r="K20" s="32" t="s">
         <v>49</v>
       </c>
-      <c r="L20" s="32" t="s">
+      <c r="L20" s="33" t="s">
         <v>50</v>
       </c>
-      <c r="M20" s="26" t="s">
+      <c r="M20" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="N20" s="32"/>
+      <c r="N20" s="33"/>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B21" s="28" t="s">
+      <c r="B21" s="29" t="s">
         <v>41</v>
       </c>
-      <c r="C21" s="28" t="s">
+      <c r="C21" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="D21" s="28" t="s">
+      <c r="D21" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="E21" s="28" t="s">
+      <c r="E21" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="F21" s="28" t="s">
+      <c r="F21" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="G21" s="3" t="s">
+      <c r="G21" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="H21" s="23" t="s">
+      <c r="H21" s="25" t="s">
         <v>60</v>
       </c>
-      <c r="I21" s="3" t="s">
+      <c r="I21" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="J21" s="24" t="n">
+      <c r="J21" s="26" t="n">
         <v>30000</v>
       </c>
-      <c r="K21" s="31" t="s">
+      <c r="K21" s="32" t="s">
         <v>49</v>
       </c>
-      <c r="L21" s="25" t="s">
+      <c r="L21" s="24" t="s">
         <v>50</v>
       </c>
-      <c r="M21" s="26" t="s">
+      <c r="M21" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="N21" s="25"/>
+      <c r="N21" s="24"/>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="27" t="s">
+      <c r="A22" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="B22" s="28" t="s">
+      <c r="B22" s="29" t="s">
         <v>41</v>
       </c>
-      <c r="C22" s="28" t="s">
+      <c r="C22" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="D22" s="28" t="s">
+      <c r="D22" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="E22" s="28" t="s">
+      <c r="E22" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="F22" s="28" t="s">
+      <c r="F22" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="G22" s="27" t="s">
+      <c r="G22" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="H22" s="29" t="s">
+      <c r="H22" s="30" t="s">
         <v>62</v>
       </c>
-      <c r="I22" s="27" t="s">
+      <c r="I22" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="J22" s="30" t="n">
+      <c r="J22" s="31" t="n">
         <v>250000</v>
       </c>
-      <c r="K22" s="31" t="s">
+      <c r="K22" s="32" t="s">
         <v>49</v>
       </c>
-      <c r="L22" s="32" t="s">
+      <c r="L22" s="33" t="s">
         <v>50</v>
       </c>
-      <c r="M22" s="26" t="s">
+      <c r="M22" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="N22" s="32"/>
+      <c r="N22" s="33"/>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="s">
+      <c r="A23" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="B23" s="28" t="s">
+      <c r="B23" s="29" t="s">
         <v>41</v>
       </c>
-      <c r="C23" s="28" t="s">
+      <c r="C23" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="D23" s="28" t="s">
+      <c r="D23" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="E23" s="28" t="s">
+      <c r="E23" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="F23" s="28" t="s">
+      <c r="F23" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="G23" s="3" t="s">
+      <c r="G23" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="H23" s="23" t="s">
+      <c r="H23" s="25" t="s">
         <v>64</v>
       </c>
-      <c r="I23" s="3" t="s">
+      <c r="I23" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="J23" s="24" t="n">
+      <c r="J23" s="26" t="n">
         <v>3000000</v>
       </c>
-      <c r="K23" s="31" t="s">
+      <c r="K23" s="32" t="s">
         <v>49</v>
       </c>
-      <c r="L23" s="25" t="s">
+      <c r="L23" s="24" t="s">
         <v>50</v>
       </c>
-      <c r="M23" s="26" t="s">
+      <c r="M23" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="N23" s="25"/>
+      <c r="N23" s="24"/>
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="27" t="s">
+      <c r="A24" s="28" t="s">
         <v>65</v>
       </c>
-      <c r="B24" s="28" t="s">
+      <c r="B24" s="29" t="s">
         <v>41</v>
       </c>
-      <c r="C24" s="28" t="s">
+      <c r="C24" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="D24" s="28" t="s">
+      <c r="D24" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="E24" s="28" t="s">
+      <c r="E24" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="F24" s="28" t="s">
+      <c r="F24" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="G24" s="27" t="s">
+      <c r="G24" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="H24" s="29" t="s">
+      <c r="H24" s="30" t="s">
         <v>66</v>
       </c>
-      <c r="I24" s="27" t="s">
+      <c r="I24" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="J24" s="30" t="n">
+      <c r="J24" s="31" t="n">
         <v>100000</v>
       </c>
-      <c r="K24" s="31" t="s">
+      <c r="K24" s="32" t="s">
         <v>49</v>
       </c>
-      <c r="L24" s="32" t="s">
+      <c r="L24" s="33" t="s">
         <v>50</v>
       </c>
-      <c r="M24" s="26" t="s">
+      <c r="M24" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="N24" s="32"/>
+      <c r="N24" s="33"/>
     </row>
   </sheetData>
   <autoFilter ref="A14:N24"/>
-  <mergeCells count="6">
-    <mergeCell ref="A1:N1"/>
-    <mergeCell ref="A2:N2"/>
-    <mergeCell ref="E4:N4"/>
-    <mergeCell ref="E5:N8"/>
-    <mergeCell ref="E10:F12"/>
-    <mergeCell ref="H10:N12"/>
-  </mergeCells>
   <hyperlinks>
     <hyperlink ref="H15" r:id="rId1" display="Site URL"/>
     <hyperlink ref="H16" r:id="rId2" display="https://immunefi.com/bug-bounty/ens/information/"/>

</xml_diff>